<commit_message>
PAUSED (task177): stage 4 round 1 fixes, waiting on round 2 readers
Round 1 on target.zip 4827dc5d: judge DETERMINISTIC (hygiene only), both readers filed the call at 10,
the asks leaked (9 of 21, 21 of 21). Ask A's primary re-sited onto the bill path: 453 app acceptances
the engine never applied are billed at the app's half-price rate with no discount line. Ask B's onto
the line path: 921 households' two same-plan subscriptions are billed on one line under the list
subscription ("x 2"). Reader B's quoted routes and both credit-note variants keep 0 of 21 in
cracker.py. Hygiene: validation floor 0.20, the plan's send date, the list's send-day name, the
credits pinned in the prompt. Call and every call-side row frozen at round 1's bytes; figures.json
unchanged. checks 141 of 141, verify 35 of 35, rebuild identical, zip cc5a56de.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task177/golden/retention_offer_forecast_2027.xlsx
+++ b/task177/golden/retention_offer_forecast_2027.xlsx
@@ -106,7 +106,7 @@
     <t>Family</t>
   </si>
   <si>
-    <t>Half-price discounts on the bills of subscriptions that took last January's offer, in the email, on the web or in the app, by the month the bill was raised; pounds to the nearest hundred. The save desk's own half price is not the offer.</t>
+    <t>Half-price discounts on the bills of subscriptions that took last January's offer, in the email, on the web or in the app, by the month the bill was raised; pounds to the nearest hundred. App acceptances the offers engine did not apply were billed at the app's half-price rate with no discount line, and are counted. The save desk's own half price is not the offer.</t>
   </si>
   <si>
     <t>October 2026 (GBP)</t>
@@ -121,7 +121,7 @@
     <t>January 2027 (GBP)</t>
   </si>
   <si>
-    <t>What the subscriptions on this year's list were billed for their plans, after credits, by the UK date each bill was raised; pounds to the nearest hundred. Each subscription's own invoice lines, on whichever account's invoice they sit; the Puzzles add-ons and other plans on the same invoices are not the list's plans.</t>
+    <t>What the subscriptions on this year's list were billed for their plans, net of credit notes and the goodwill credits on its invoices, by the UK date each bill was raised; pounds to the nearest hundred. Each subscription's own invoice lines, on whichever account's invoice they sit, a line billing two subscriptions of a household counted once; the Puzzles add-ons and other plans on the same invoices are not the list's plans.</t>
   </si>
   <si>
     <t>As of</t>

</xml_diff>